<commit_message>
added musc for osc
</commit_message>
<xml_diff>
--- a/library/diode.xlsx
+++ b/library/diode.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitProjects\elem_altium_db2\library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0103C903-9CA8-4938-9853-D3FC3534B62C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F743DC30-A8CE-4209-A12C-E15E9369AE7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{EE2E7F00-6B54-4C0B-98D7-835E87062BAF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{EE2E7F00-6B54-4C0B-98D7-835E87062BAF}"/>
   </bookViews>
   <sheets>
     <sheet name="array" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="83">
   <si>
     <t>Part Number</t>
   </si>
@@ -278,6 +278,12 @@
   </si>
   <si>
     <t>SMC</t>
+  </si>
+  <si>
+    <t>ESD9L5.0ST5G</t>
+  </si>
+  <si>
+    <t>ESD9L5.0ST5G SOD-923</t>
   </si>
 </sst>
 </file>
@@ -713,8 +719,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E834B2D-3CFC-49B2-A2B4-67F2231F306F}">
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="19.42578125" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" customWidth="1"/>
+    <col min="3" max="3" width="36.140625" customWidth="1"/>
+    <col min="4" max="4" width="20" customWidth="1"/>
+    <col min="5" max="5" width="24.42578125" customWidth="1"/>
+    <col min="6" max="6" width="19" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -1130,6 +1144,29 @@
         <v>13</v>
       </c>
     </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>81</v>
+      </c>
+      <c r="B19" t="s">
+        <v>72</v>
+      </c>
+      <c r="C19" t="s">
+        <v>82</v>
+      </c>
+      <c r="D19" t="s">
+        <v>81</v>
+      </c>
+      <c r="E19" t="s">
+        <v>17</v>
+      </c>
+      <c r="F19" t="s">
+        <v>74</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
new for mr bakaev
</commit_message>
<xml_diff>
--- a/library/diode.xlsx
+++ b/library/diode.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitProjects\elem_altium_db2\library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97A50066-EBF2-4280-B324-DF3BA9362278}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{187C824A-4370-4266-AEE4-975EF662CBB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1425" yWindow="1425" windowWidth="23085" windowHeight="13635" xr2:uid="{EE2E7F00-6B54-4C0B-98D7-835E87062BAF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{EE2E7F00-6B54-4C0B-98D7-835E87062BAF}"/>
   </bookViews>
   <sheets>
     <sheet name="array" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="119">
   <si>
     <t>Part Number</t>
   </si>
@@ -389,6 +389,9 @@
   </si>
   <si>
     <t>аА0.339.583ТУ</t>
+  </si>
+  <si>
+    <t>SOD123W</t>
   </si>
 </sst>
 </file>
@@ -445,12 +448,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Accent 3 2" xfId="1" xr:uid="{07D6D35A-A25D-4183-ACA2-756DA14CBAEA}"/>
@@ -915,7 +917,7 @@
       <c r="F6" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" t="s">
         <v>117</v>
       </c>
     </row>
@@ -926,7 +928,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E834B2D-3CFC-49B2-A2B4-67F2231F306F}">
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.42578125" customWidth="1"/>
@@ -1556,6 +1558,26 @@
         <v>113</v>
       </c>
     </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>50</v>
+      </c>
+      <c r="C28" t="s">
+        <v>50</v>
+      </c>
+      <c r="D28" t="s">
+        <v>50</v>
+      </c>
+      <c r="E28" t="s">
+        <v>45</v>
+      </c>
+      <c r="F28" t="s">
+        <v>118</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>